<commit_message>
Added new RDF data schemes and visual schemes for economy-table85-89, and fixed XLSX spreadsheets for economy-table86-87
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table86.xlsx
+++ b/sources/table_normalization/xlsx/economy-table86.xlsx
@@ -195,7 +195,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -240,7 +240,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -346,49 +346,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment indent="2"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment indent="3"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment indent="4"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment indent="2"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -401,15 +388,35 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -718,94 +725,94 @@
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="13"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="13" t="s">
+      <c r="J1" s="24"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="15"/>
-      <c r="N1" s="16"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="27"/>
     </row>
     <row r="2" spans="1:14" ht="13">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18" t="s">
+      <c r="A2" s="21"/>
+      <c r="B2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="20"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="20" t="s">
+      <c r="J2" s="15"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="20"/>
-      <c r="N2" s="21"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="16"/>
     </row>
     <row r="3" spans="1:14" ht="13">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="23" t="s">
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="24" t="s">
+      <c r="K3" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="23" t="s">
+      <c r="L3" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="M3" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="24" t="s">
+      <c r="N3" s="29" t="s">
         <v>13</v>
       </c>
     </row>
@@ -854,22 +861,22 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="26"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="23"/>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
@@ -916,22 +923,22 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="26"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="23"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3" t="s">
@@ -1374,22 +1381,22 @@
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="25"/>
-      <c r="M18" s="25"/>
-      <c r="N18" s="26"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="23"/>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="4" t="s">

</xml_diff>

<commit_message>
Fixed economy-table86 and 96 spreadsheets, economy-table88.ttl
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table86.xlsx
+++ b/sources/table_normalization/xlsx/economy-table86.xlsx
@@ -346,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -373,9 +373,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -399,12 +396,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
@@ -416,6 +407,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -725,94 +722,94 @@
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="24"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="12" t="s">
+      <c r="J1" s="27"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="26"/>
-      <c r="N1" s="27"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="24"/>
     </row>
     <row r="2" spans="1:14" ht="13">
-      <c r="A2" s="21"/>
-      <c r="B2" s="13" t="s">
+      <c r="A2" s="20"/>
+      <c r="B2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="15" t="s">
+      <c r="J2" s="14"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="N2" s="16"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="15"/>
     </row>
     <row r="3" spans="1:14" ht="13">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="28" t="s">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="29" t="s">
+      <c r="K3" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="28" t="s">
+      <c r="L3" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="28" t="s">
+      <c r="M3" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="29" t="s">
+      <c r="N3" s="26" t="s">
         <v>13</v>
       </c>
     </row>
@@ -861,22 +858,22 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="23"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="22"/>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
@@ -923,22 +920,22 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="23"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="22"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3" t="s">
@@ -1381,22 +1378,22 @@
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="23"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="22"/>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="4" t="s">

</xml_diff>